<commit_message>
CAR Varones: metrado sin las referencias a las laminas excluidas (DP-08, DA-01 a DA-03); cantidades sin cambio
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables_varones/METRADO_DRENAJE_PLUVIAL_CAR_VARONES_23-10-2026.xlsx
+++ b/entregables_varones/METRADO_DRENAJE_PLUVIAL_CAR_VARONES_23-10-2026.xlsx
@@ -2080,60 +2080,60 @@
     <t>Sobreancho de excavacion a cada lado del colector</t>
   </si>
   <si>
-    <t>Laminas DPLV-21 y DPLV-22: zanja de 1.40 m (0.90 + 2 x 0.25)</t>
+    <t>Zanja de 1.40 m (0.90 + 2 x 0.25)</t>
   </si>
   <si>
     <t>Franja de relleno de nivelacion del retiro, lado via</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
+    <t>Recubrimiento del acero</t>
+  </si>
+  <si>
+    <t>Norma E.060, tabla 7.7.1 (concreto en contacto con el suelo)</t>
+  </si>
+  <si>
+    <t>Peso de la barra de 3/8"</t>
+  </si>
+  <si>
+    <t>Igual a PARAMETROS!B10 de esta planilla</t>
+  </si>
+  <si>
+    <t>Peso de la barra de 1/2"</t>
+  </si>
+  <si>
+    <t>Catalogo del fabricante (0.994 kg/m)</t>
+  </si>
+  <si>
+    <t>Traslape de barras longitudinales</t>
+  </si>
+  <si>
+    <t>Norma E.060, 12.15 (clase B, 3/8"): 0.40 m</t>
+  </si>
+  <si>
+    <t>Longitud comercial de barra</t>
+  </si>
+  <si>
+    <t>Igual a PARAMETROS!B11 de esta planilla</t>
+  </si>
+  <si>
+    <t>Ganchos de cierre del marco (2 x 0.15)</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Igual a PARAMETROS!B16 de esta planilla</t>
+  </si>
+  <si>
+    <t>Espaciamiento de marcos en tramo normal</t>
+  </si>
+  <si>
     <t>Laminas DPLV-21 y DPLV-22</t>
   </si>
   <si>
-    <t>Recubrimiento del acero</t>
-  </si>
-  <si>
-    <t>Norma E.060, tabla 7.7.1 (concreto en contacto con el suelo)</t>
-  </si>
-  <si>
-    <t>Peso de la barra de 3/8"</t>
-  </si>
-  <si>
-    <t>Igual a PARAMETROS!B10 de esta planilla</t>
-  </si>
-  <si>
-    <t>Peso de la barra de 1/2"</t>
-  </si>
-  <si>
-    <t>Catalogo del fabricante (0.994 kg/m)</t>
-  </si>
-  <si>
-    <t>Traslape de barras longitudinales</t>
-  </si>
-  <si>
-    <t>Norma E.060, 12.15 (clase B, 3/8"): 0.40 m</t>
-  </si>
-  <si>
-    <t>Longitud comercial de barra</t>
-  </si>
-  <si>
-    <t>Igual a PARAMETROS!B11 de esta planilla</t>
-  </si>
-  <si>
-    <t>Ganchos de cierre del marco (2 x 0.15)</t>
-  </si>
-  <si>
-    <t>Laminas DPLV-21 y DPLV-22, armadura</t>
-  </si>
-  <si>
-    <t>Igual a PARAMETROS!B16 de esta planilla</t>
-  </si>
-  <si>
-    <t>Espaciamiento de marcos en tramo normal</t>
-  </si>
-  <si>
-    <t>Laminas DPLV-21 y DPLV-22</t>
-  </si>
-  <si>
     <t>Espaciamiento de marcos en el cruce de camiones</t>
   </si>
   <si>
@@ -2209,7 +2209,7 @@
     <t>COLECTOR PLUVIAL FRONTAL - METRADO DE MOVIMIENTO DE TIERRAS</t>
   </si>
   <si>
-    <t>Criterio (laminas DPLV-21 y DPLV-22): LIMPIEZA Y TRAZO = ancho de zanja x L.  EXCAVACION = ancho de zanja x Hz x L, con Hz = terreno existente (topografia) - fondo del solado.  REFINE = (ancho exterior + 0.10) x L (fondo del solado).  RELLENO LATERAL = 2 x sobreancho x Hz x L.  RELLENO FRANJA = 1.00 x (NPT - terreno) x L (nivelacion del retiro lado via).  h y Hz son valores medios ponderados del tramo (perfil DPLV-18 y topografia); el detalle cada 2.00 m esta en la memoria de calculo.</t>
+    <t>Criterio: LIMPIEZA Y TRAZO = ancho de zanja x L.  EXCAVACION = ancho de zanja x Hz x L, con Hz = terreno existente (topografia) - fondo del solado.  REFINE = (ancho exterior + 0.10) x L (fondo del solado).  RELLENO LATERAL = 2 x sobreancho x Hz x L.  RELLENO FRANJA = 1.00 x (NPT - terreno) x L (nivelacion del retiro lado via).  h y Hz son valores medios ponderados del tramo (perfil DPLV-18 y topografia); el detalle cada 2.00 m esta en la memoria de calculo.</t>
   </si>
   <si>
     <t>ZONA</t>
@@ -2266,7 +2266,7 @@
     <t>0+006.08</t>
   </si>
   <si>
-    <t>DPLV-17 (planta), DPLV-18 (perfil: fondo y terreno), DPLV-21 y DPLV-22 (seccion y criterio)</t>
+    <t>DPLV-17 (planta), DPLV-18 (perfil: fondo y terreno), DPLV-21 y DPLV-22 (seccion)</t>
   </si>
   <si>
     <t>tramo normal</t>
@@ -2311,7 +2311,7 @@
     <t>COLECTOR PLUVIAL FRONTAL - METRADO DE CONCRETO SIMPLE Y ARMADO</t>
   </si>
   <si>
-    <t>Criterio (laminas DPLV-21 y DPLV-22): SOLADO = (ancho exterior + 0.10) x L.  LOSA DE FONDO = ancho exterior x e fondo x L.  MUROS = 2 x e muro x h x L.  LOSA SUPERIOR = ancho exterior x e losa x L.  ACABADO = ancho exterior x L (losa superior frotachada y brunada).  CURADO = 2 caras interiores de muros (2 x h x L) + fondo interior (b x L) + losa superior (ancho exterior x L), igual al criterio de la hoja METRADO DE CURADO.</t>
+    <t>Criterio: SOLADO = (ancho exterior + 0.10) x L.  LOSA DE FONDO = ancho exterior x e fondo x L.  MUROS = 2 x e muro x h x L.  LOSA SUPERIOR = ancho exterior x e losa x L.  ACABADO = ancho exterior x L (losa superior frotachada y brunada).  CURADO = 2 caras interiores de muros (2 x h x L) + fondo interior (b x L) + losa superior (ancho exterior x L), igual al criterio de la hoja METRADO DE CURADO.</t>
   </si>
   <si>
     <t>ANCHO EXT. (m)</t>
@@ -2335,7 +2335,7 @@
     <t>CURADO (m2)</t>
   </si>
   <si>
-    <t>DPLV-21 y DPLV-22 (secciones y areas por metro), DPLV-18 (h por tramo)</t>
+    <t>DPLV-21 y DPLV-22 (secciones), DPLV-18 (h por tramo)</t>
   </si>
   <si>
     <t>TOTAL COLECTOR (tramos)</t>
@@ -2392,7 +2392,7 @@
     <t>COLECTOR PLUVIAL FRONTAL - METRADO DE ENCOFRADO Y DESENCOFRADO</t>
   </si>
   <si>
-    <t>Criterio (laminas DPLV-21 y DPLV-22): se encofran las dos caras interiores de los muros, las dos caras exteriores en toda la altura del cajon (losa de fondo + muro + losa superior) y el fondo de la losa superior (ancho interior b). La losa de fondo se vacia sobre el solado y la cara superior de la losa queda libre (acabado).</t>
+    <t>Criterio: se encofran las dos caras interiores de los muros, las dos caras exteriores en toda la altura del cajon (losa de fondo + muro + losa superior) y el fondo de la losa superior (ancho interior b). La losa de fondo se vacia sobre el solado y la cara superior de la losa queda libre (acabado).</t>
   </si>
   <si>
     <t>ANCHO INT. b (m)</t>
@@ -2410,7 +2410,7 @@
     <t>TOTAL ENCOFRADO (m2)</t>
   </si>
   <si>
-    <t>DPLV-21 y DPLV-22 (secciones y areas por metro)</t>
+    <t>DPLV-21 y DPLV-22 (secciones)</t>
   </si>
   <si>
     <t>RESUMEN PARA LA PLANILLA GENERAL (partida 01.04.04.04.04)</t>
@@ -2464,10 +2464,10 @@
     <t>TOTAL (kg)</t>
   </si>
   <si>
-    <t>DPLV-21 (seccion S-01; armadura)</t>
-  </si>
-  <si>
-    <t>DPLV-21 y DPLV-22 (secciones S-02 a S-08; armadura)</t>
+    <t>DPLV-21 (seccion S-01)</t>
+  </si>
+  <si>
+    <t>DPLV-21 y DPLV-22 (seccion S-02 a S-08)</t>
   </si>
   <si>
     <t>DIAM.</t>

</xml_diff>